<commit_message>
1.选题—开题报告\参考论文(已自动还原).xlsx 2.开题报告\模版\CN（翻译版）_Appendix-1-Form for the registration of the subject .docx 2.开题报告\实稿\Appendix-Form for the registration of the subject（最终递交版本）-1788788149546.docx 2.开题报告\实稿\CN（翻译版）_Appendix-1-Form for the registration of the subject.docx
Signed-off-by: 徐振宇 <xuzhenyu3333@gmail.com>
</commit_message>
<xml_diff>
--- a/1.选题—开题报告/参考论文(已自动还原).xlsx
+++ b/1.选题—开题报告/参考论文(已自动还原).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UMEF毕业\1.选题—开题报告\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C4AAA4-75B8-44B6-B431-8AF265FEEF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E94AB9-03E2-43F3-B574-B337F6D3E8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28575" yWindow="3315" windowWidth="28800" windowHeight="15090" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28695" yWindow="2970" windowWidth="28800" windowHeight="15090" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="跌倒预测" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>[1]高伊楠,张乾龙,党冉冉,等.社区老年糖尿病患者跌倒风险预测模型的构建[J].牡丹江医科大学学报,2026,47(2):27-31.DOI:10.13799/j.cnki.mdjyxyxb.2026.02.001.</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -64,10 +64,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>列1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>老年康复科护理文书</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -113,6 +109,49 @@
   </si>
   <si>
     <t>4.基于预训练模型的护理文书缺陷自动检测与质控系统研究</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>质控小组干预下肿瘤科护理病历书写质量的效果观察</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kns.cnki.net/kcms2/article/abstract?v=HTCMX8yYpPFOCJhPua_vh148WzWpqAF_LwNeDWQzGIj0XCJdwVHGdwc1ez2yTagB4b3Kajq2YpwNTKwIu459k_GvFW3yTd7qoVnuVXAk0nG_c9mi7GwWYeC59MzwW-pOdfOfCardjbRotcdsm4igf9GOycKIMsNJudvkuI0-Aw1T3sMNQKT0rg==&amp;uniplatform=NZKPT&amp;language=CHS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PDCA在儿科护理文书书写质量管理的应用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目的 采用PDCA模式对儿科护理文书书写进行质量管理，提高护理文书书写质量，保障医疗安全。方法 随机抽取2018年1月1日-2018年12月31日某院小儿内分泌科60例患儿的护理文书作为对照组，对其书写质量进行质量监控，开展PDCA循环管理,随机抽取实施改进措施后的2019年1月1日-2019年12月31日60例患儿的护理文书作为观察组。比较2组护理文书书写质量，并进行评价。结果 观察组护理文书质量评分(97.62±3.93)分高于对照组护理的(92.59±3.74)分，两组比较差异具有统计学意义，P&lt;0.05。观察组各种风险评估不合格(6.67%)、护理记录缺项、漏项、记录不完整(3.33%)、护理记录复制(3.33%)、病情动态评估与描述不准确(5.00%)、与医师记录不一致(3.33%)及未体现专科特色(3.33%)的发生率与对照组(40.00%、15.00%、16.67%、20.00%、16.67%、36.67%)比较显著减少，差异具有统计学意义(P&lt;0.05)，合格率(96.67%)与对照组(90.00%)比较显著升高，差异具有统计学意义，(P&lt;0.05)。结论 PDCA模式在护理文书书写质量管理中，能够降低护理文书书写错误率，提高某院内分泌科护理文书书写质量及合格率。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>摘要</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kns.cnki.net/kcms2/article/abstract?v=tBI8TAhqnxQlGVA1mSoZnDn2Nt2nYOLfhBFOh8p5Xq6T3LnGa0rfKB-_DB2gK5OtIeIJHldPxlrzA8KTbwF7ip4OgwNkIQjA40kB28KyNbKSIyRipD5Mj96EYJJgS4Hexhm2aS-l-26tHLjVg03olIp1o1ib39c7HYXdXcfRKd4_KCKADzEKDQ==&amp;uniplatform=NZKPT&amp;language=CHS</t>
+  </si>
+  <si>
+    <t>文章相关内容</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PDCA 能对护理文书书写质量产生较好质控效果。与杨燕等[8]研究结果比较，本研究应用的 PDCA 管理对儿科护理文书质量的改善效果更明显。研究中观察组各种风险评估不合格(6.67%) 、 护 理 记 录 缺 项 、 漏 项 、 记 录 不 完 整(3.33%)、护理记录复制(3.33%)、病情动态评估与 描 述 不 准 确 (5.00%) 、 与 医 师 记 录 不 一 致(3.33%)及未体现专科特色</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>基于Flask的单病种上报AI平台的设计与实现</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://kns.cnki.net/kcms2/article/abstract?v=tBI8TAhqnxTaPq8iz5oQOiMRZmUYBit6nSJF2FwE_cl5xGiQCfCgvsoztgMQzxTGM-PQ_49RZQcCX5V5FoTF6rAaHcUiSmvMEULM1QKjmoNRFOkvkieq-TO5u6a1_sxu9Cyg9GMgkZZCkYHfdn_RjkPh2AYJmpF0hyon0mzvwnlDRAAScZqVIhlNMf_976z_&amp;uniplatform=NZKPT&amp;language=CHS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>近些年来,随着疾病谱的日益复杂变化和广大人民群众对高质量医疗服务的要求,国家卫健委已出台系列管理工作规划,专注于实现我国医疗质量安全管理工作更加科学、精细。在国家卫健委逐步优化和健全单病种体系后,进一步扩大了我国单病种质控范围,单病种疾病数量增加到51个,涵盖了心血管疾病、神经系统疾病、呼吸系统疾病、生殖系统疾病以及眼科口腔系统等多个方面的疾病,单病种指标项更是达到了7000余项。这给卫生健康行政部门、医疗机构、质控中心对单病种进行质量管理与控制带来了巨大的挑战。 本研究分析了国内某三级医院单病种管理与控制工作中单病种上报的现状,归纳当前医院单病种上报工作的重点和医生进行单病种上报工作中遇到的难点,总结出上报医生对单病种上报的功能与性能需求,开发了基于Flask的单病种上报AI平台。平台采用了B/S模式,整合了Flask和Vue两个框架以及Chinese-roberta-wwm-ext模型,完成了首页统计数据可视化展示、智能填报、上报分析、用户管理等四个功能模块。其中,首页可视化展示使用Echarts图表库,后台单病种上报接口使用正则匹配技术和自然语言处理(natural language processing,NLP)技术实现对单病种上报项的提取。采用UML统一建模语言,使用用例图分析单病种上报的业务需求,并通过类图和时序图对系统进行静态与动态建模设计。最后在系统测试阶段,对上报AI平台的主要功能进行测试。 单病种体系庞大,管理与控制工作复杂,开发出满足上报工作需求的平台,自动提取上报项并填充填报页面,避免上报医生逐项地填写上报项内容,将提高单病种的上报效率,节约医疗成本,最终提升医院乃至国家对单病种质量的管理与控制的能力。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -120,7 +159,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,6 +180,22 @@
       <color theme="10"/>
       <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -165,7 +220,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -182,13 +237,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="等线"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </font>
       <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -641,12 +722,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3EA2BE98-62AC-47AF-A96A-191860087D75}" name="表1" displayName="表1" ref="A1:C2" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="A1:C2" xr:uid="{3EA2BE98-62AC-47AF-A96A-191860087D75}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{7ED9AEC6-5955-4690-AC13-E153C97C2C72}" name="论文引用" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{AB05E964-C40D-4933-8E1A-D53A4927A43D}" name="链接" dataDxfId="1" dataCellStyle="超链接"/>
-    <tableColumn id="3" xr3:uid="{28314E1D-97D5-4298-BC22-6CADD539BAF1}" name="列1" dataDxfId="0" dataCellStyle="超链接"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3EA2BE98-62AC-47AF-A96A-191860087D75}" name="表1" displayName="表1" ref="A1:D5" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D5" xr:uid="{3EA2BE98-62AC-47AF-A96A-191860087D75}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{7ED9AEC6-5955-4690-AC13-E153C97C2C72}" name="论文引用" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{AB05E964-C40D-4933-8E1A-D53A4927A43D}" name="链接" dataDxfId="2" dataCellStyle="超链接"/>
+    <tableColumn id="3" xr3:uid="{28314E1D-97D5-4298-BC22-6CADD539BAF1}" name="摘要" dataDxfId="1" dataCellStyle="超链接"/>
+    <tableColumn id="4" xr3:uid="{255DA137-3FE7-463B-BD85-87BE53A31A72}" name="文章相关内容" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -947,26 +1029,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99949835-AFA3-48A3-A383-A6D26E385748}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.125" style="1" customWidth="1"/>
     <col min="2" max="2" width="78" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28" style="5" customWidth="1"/>
+    <col min="3" max="3" width="73.25" style="8" customWidth="1"/>
+    <col min="4" max="4" width="50.25" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
+      <c r="C1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="3" customFormat="1" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" s="3" customFormat="1" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -976,15 +1062,55 @@
       <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" spans="1:4" ht="81" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" spans="1:4" ht="201.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{C09D4A3E-F77C-4F6E-9E0C-8B09F7447FE6}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://kns.cnki.net/kcms2/article/abstract?v=2g3PLS-OwFpRXgll7tj3ZQjah-o_hH0bm9xu-f2kPDMZJgN-HUDDqcHUCrac9tQqfBy08Pv34h6zXQwAbWZ6pIGRX1aa8pN7Ffj1a22PfKljng1Zp1x-bHNeaUhxYztXcOCbjWiRaTend8TK3nUO7XrWsjIlxAUdDpA25drhP82keBfJB28bT3ZkwL6egjre&amp;uniplatform=NZKPT&amp;language=CHS" xr:uid="{39CE76DE-1345-4503-B7EB-271451CB2C80}"/>
+    <hyperlink ref="B3" r:id="rId3" display="https://kns.cnki.net/kcms2/article/abstract?v=HTCMX8yYpPFOCJhPua_vh148WzWpqAF_LwNeDWQzGIj0XCJdwVHGdwc1ez2yTagB4b3Kajq2YpwNTKwIu459k_GvFW3yTd7qoVnuVXAk0nG_c9mi7GwWYeC59MzwW-pOdfOfCardjbRotcdsm4igf9GOycKIMsNJudvkuI0-Aw1T3sMNQKT0rg==&amp;uniplatform=NZKPT&amp;language=CHS" xr:uid="{112C404C-10DB-46AD-AAF0-9599A18831BC}"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://kns.cnki.net/kcms2/article/abstract?v=tBI8TAhqnxTaPq8iz5oQOiMRZmUYBit6nSJF2FwE_cl5xGiQCfCgvsoztgMQzxTGM-PQ_49RZQcCX5V5FoTF6rAaHcUiSmvMEULM1QKjmoNRFOkvkieq-TO5u6a1_sxu9Cyg9GMgkZZCkYHfdn_RjkPh2AYJmpF0hyon0mzvwnlDRAAScZqVIhlNMf_976z_&amp;uniplatform=NZKPT&amp;language=CHS" xr:uid="{238BCE44-5C82-4949-93ED-21FEFADD3F21}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1001,46 +1127,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>